<commit_message>
Finalize D2 strict and sensitive availability assessment
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_Fig05_source_data.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/data/D2_Fig05_source_data.xlsx
@@ -552,11 +552,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>info_empty_cov</t>
+          <t>hard_stasis_fraction_observed</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.3847410553831073</v>
+        <v>0.01198452906248298</v>
       </c>
     </row>
     <row r="9">
@@ -567,11 +567,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>info_empty_cov</t>
+          <t>hard_stasis_fraction_observed</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.6246256058378261</v>
+        <v>0.2543988669172523</v>
       </c>
     </row>
   </sheetData>
@@ -5125,7 +5125,7 @@
         <v>45882</v>
       </c>
       <c r="B14" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -5136,10 +5136,10 @@
         <v>45883</v>
       </c>
       <c r="B15" t="n">
-        <v>0.4166666666666667</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.4166666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -5147,10 +5147,10 @@
         <v>45884</v>
       </c>
       <c r="B16" t="n">
-        <v>9.027777777777777</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>8.611111111111112</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -5367,10 +5367,10 @@
         <v>45904</v>
       </c>
       <c r="B36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -5455,10 +5455,10 @@
         <v>45912</v>
       </c>
       <c r="B44" t="n">
-        <v>25.20833333333333</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>25.34722222222222</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -5788,7 +5788,7 @@
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -5807,7 +5807,7 @@
         <v>45944</v>
       </c>
       <c r="B76" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C76" t="n">
         <v>0</v>
@@ -5818,10 +5818,10 @@
         <v>45945</v>
       </c>
       <c r="B77" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -5840,10 +5840,10 @@
         <v>45947</v>
       </c>
       <c r="B79" t="n">
-        <v>0.1157407407407408</v>
+        <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -5851,7 +5851,7 @@
         <v>45948</v>
       </c>
       <c r="B80" t="n">
-        <v>0.02314814814814815</v>
+        <v>0</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
@@ -5873,10 +5873,10 @@
         <v>45950</v>
       </c>
       <c r="B82" t="n">
-        <v>0.01157407407407408</v>
+        <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -5884,7 +5884,7 @@
         <v>45951</v>
       </c>
       <c r="B83" t="n">
-        <v>0.05787037037037038</v>
+        <v>0</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -5898,7 +5898,7 @@
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -5906,7 +5906,7 @@
         <v>45953</v>
       </c>
       <c r="B85" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
       <c r="C85" t="n">
         <v>0</v>
@@ -5920,7 +5920,7 @@
         <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -5939,10 +5939,10 @@
         <v>45956</v>
       </c>
       <c r="B88" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
@@ -5950,7 +5950,7 @@
         <v>45957</v>
       </c>
       <c r="B89" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C89" t="n">
         <v>0</v>
@@ -5964,7 +5964,7 @@
         <v>0</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02314814814814815</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -5972,10 +5972,10 @@
         <v>45959</v>
       </c>
       <c r="B91" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>0.1157407407407408</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -6005,10 +6005,10 @@
         <v>45962</v>
       </c>
       <c r="B94" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
       <c r="C94" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -6203,10 +6203,10 @@
         <v>45980</v>
       </c>
       <c r="B112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -6214,10 +6214,10 @@
         <v>45981</v>
       </c>
       <c r="B113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -6731,10 +6731,10 @@
         <v>46028</v>
       </c>
       <c r="B160" t="n">
-        <v>36.21527777777778</v>
+        <v>0</v>
       </c>
       <c r="C160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -6742,10 +6742,10 @@
         <v>46029</v>
       </c>
       <c r="B161" t="n">
-        <v>3.993055555555555</v>
+        <v>0</v>
       </c>
       <c r="C161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -7798,10 +7798,10 @@
         <v>46125</v>
       </c>
       <c r="B257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="C257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8154,22 +8154,22 @@
         <v>45883</v>
       </c>
       <c r="B15" t="n">
-        <v>0.3472222222222222</v>
+        <v>0</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3472222222222222</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>0.3993055555555556</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3472222222222222</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0.3472222222222222</v>
+        <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3645833333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -8177,22 +8177,22 @@
         <v>45884</v>
       </c>
       <c r="B16" t="n">
-        <v>8.888888888888889</v>
+        <v>0</v>
       </c>
       <c r="C16" t="n">
-        <v>8.680555555555557</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>9.097222222222221</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>8.912037037037038</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>8.767361111111111</v>
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>9.02199074074074</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -8637,22 +8637,22 @@
         <v>45904</v>
       </c>
       <c r="B36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="C36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2083333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -8821,22 +8821,22 @@
         <v>45912</v>
       </c>
       <c r="B44" t="n">
-        <v>25.3125</v>
+        <v>0</v>
       </c>
       <c r="C44" t="n">
-        <v>25.20833333333333</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>25.41666666666667</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>25.27777777777778</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>25.20833333333333</v>
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>25.39930555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -9540,7 +9540,7 @@
         <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>0.02604166666666667</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
@@ -9557,13 +9557,13 @@
         <v>45944</v>
       </c>
       <c r="B76" t="n">
-        <v>0.01736111111111111</v>
+        <v>0</v>
       </c>
       <c r="C76" t="n">
         <v>0</v>
       </c>
       <c r="D76" t="n">
-        <v>0.0607638888888889</v>
+        <v>0</v>
       </c>
       <c r="E76" t="n">
         <v>0</v>
@@ -9586,7 +9586,7 @@
         <v>0</v>
       </c>
       <c r="D77" t="n">
-        <v>0.06944444444444445</v>
+        <v>0</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
@@ -9595,7 +9595,7 @@
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>0.05208333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -9609,7 +9609,7 @@
         <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>0.03472222222222222</v>
+        <v>0</v>
       </c>
       <c r="E78" t="n">
         <v>0</v>
@@ -9618,7 +9618,7 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>0.03472222222222222</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -9649,13 +9649,13 @@
         <v>45948</v>
       </c>
       <c r="B80" t="n">
-        <v>0.01736111111111111</v>
+        <v>0</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
       </c>
       <c r="D80" t="n">
-        <v>0.0607638888888889</v>
+        <v>0</v>
       </c>
       <c r="E80" t="n">
         <v>0</v>
@@ -9701,7 +9701,7 @@
         <v>0</v>
       </c>
       <c r="D82" t="n">
-        <v>0.008680555555555556</v>
+        <v>0</v>
       </c>
       <c r="E82" t="n">
         <v>0</v>
@@ -9764,13 +9764,13 @@
         <v>45953</v>
       </c>
       <c r="B85" t="n">
-        <v>0.01157407407407408</v>
+        <v>0</v>
       </c>
       <c r="C85" t="n">
         <v>0</v>
       </c>
       <c r="D85" t="n">
-        <v>0.05787037037037038</v>
+        <v>0</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
@@ -9787,13 +9787,13 @@
         <v>45954</v>
       </c>
       <c r="B86" t="n">
-        <v>0.02314814814814815</v>
+        <v>0</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
       </c>
       <c r="D86" t="n">
-        <v>0.06365740740740741</v>
+        <v>0</v>
       </c>
       <c r="E86" t="n">
         <v>0</v>
@@ -9871,7 +9871,7 @@
         <v>0</v>
       </c>
       <c r="G89" t="n">
-        <v>0.05208333333333334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -10385,22 +10385,22 @@
         <v>45980</v>
       </c>
       <c r="B112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="C112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="D112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="E112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="F112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
       <c r="G112" t="n">
-        <v>1.180555555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -10408,22 +10408,22 @@
         <v>45981</v>
       </c>
       <c r="B113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="C113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="D113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="E113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="F113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
       <c r="G113" t="n">
-        <v>0.1388888888888889</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -11489,22 +11489,22 @@
         <v>46028</v>
       </c>
       <c r="B160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
       <c r="C160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
       <c r="D160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
       <c r="E160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
       <c r="F160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
       <c r="G160" t="n">
-        <v>36.18055555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161">
@@ -11512,22 +11512,22 @@
         <v>46029</v>
       </c>
       <c r="B161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
       <c r="C161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
       <c r="D161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
       <c r="E161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
       <c r="F161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
       <c r="G161" t="n">
-        <v>3.958333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162">
@@ -13720,22 +13720,22 @@
         <v>46125</v>
       </c>
       <c r="B257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="C257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="D257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="E257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="F257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
       <c r="G257" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>